<commit_message>
added pick and choose menu
</commit_message>
<xml_diff>
--- a/data/TCI_Banquet_Grid.xlsx
+++ b/data/TCI_Banquet_Grid.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8938B67A-F69E-4450-8EE4-AAAA2C9FC7D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C684D827-DCE6-4068-BC1A-5BE618DC6FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
   <si>
     <t>Salads</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>4. In Gold (Main Course) will have set of 2 Cuisines and Platinum to have 3 Cuisines</t>
+  </si>
+  <si>
+    <t>Menu Types</t>
   </si>
 </sst>
 </file>
@@ -611,7 +614,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -623,12 +626,11 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -659,7 +661,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -690,11 +692,21 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -724,17 +736,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -760,9 +762,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -800,9 +802,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -835,26 +837,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -887,26 +872,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1081,1016 +1049,1023 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I46"/>
-  <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.5703125" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.08984375" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-    </row>
-    <row r="2" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="38"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-    </row>
-    <row r="3" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="38"/>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="38"/>
-    </row>
-    <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="38"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
-      <c r="G4" s="38"/>
-      <c r="H4" s="38"/>
-      <c r="I4" s="38"/>
-    </row>
-    <row r="5" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="39"/>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="39"/>
-    </row>
-    <row r="6" spans="1:9" s="9" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="10"/>
-      <c r="B6" s="14" t="s">
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+    </row>
+    <row r="2" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="41"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+    </row>
+    <row r="3" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="41"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+    </row>
+    <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="41"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+    </row>
+    <row r="5" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="42"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+    </row>
+    <row r="6" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="25" t="s">
+      <c r="I6" s="24" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="10"/>
-      <c r="B7" s="15" t="s">
+    <row r="7" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9"/>
+      <c r="B7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="H7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="26" t="s">
+      <c r="I7" s="25" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="14">
         <v>1200</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="25">
         <v>1350</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="14">
         <v>1350</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="25">
         <v>1500</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="14">
         <v>1900</v>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="25">
         <v>2200</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="14">
         <v>2500</v>
       </c>
-      <c r="I8" s="26">
+      <c r="I8" s="25">
         <v>2800</v>
       </c>
     </row>
-    <row r="9" spans="1:9" s="12" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" s="11" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="15">
         <v>1000</v>
       </c>
-      <c r="C9" s="27">
+      <c r="C9" s="26">
         <v>1150</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="15">
         <v>1200</v>
       </c>
-      <c r="E9" s="27">
+      <c r="E9" s="26">
         <v>1350</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="15">
         <v>1750</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="26">
         <v>2000</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9" s="15">
         <v>2300</v>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="26">
         <v>2600</v>
       </c>
     </row>
-    <row r="10" spans="1:9" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
+    <row r="10" spans="1:9" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="14">
         <v>800</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="36">
         <v>950</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="14">
         <v>1000</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="36">
         <v>1150</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="14">
         <v>1650</v>
       </c>
-      <c r="G10" s="37">
+      <c r="G10" s="36">
         <v>1850</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="14">
         <v>2100</v>
       </c>
-      <c r="I10" s="37">
+      <c r="I10" s="36">
         <v>2500</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:9" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="17">
         <v>100</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="27">
         <v>100</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="17">
         <v>150</v>
       </c>
-      <c r="E11" s="28">
+      <c r="E11" s="27">
         <v>150</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="17">
         <v>200</v>
       </c>
-      <c r="G11" s="28">
+      <c r="G11" s="27">
         <v>200</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="17">
         <v>300</v>
       </c>
-      <c r="I11" s="28">
+      <c r="I11" s="27">
         <v>300</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="40"/>
-      <c r="B12" s="41"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="41"/>
-      <c r="I12" s="41"/>
-    </row>
-    <row r="13" spans="1:9" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="42" t="s">
+    <row r="12" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="43"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+    </row>
+    <row r="13" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="44"/>
-    </row>
-    <row r="14" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="46"/>
+      <c r="I13" s="47"/>
+    </row>
+    <row r="14" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="17">
-        <v>0</v>
-      </c>
-      <c r="C14" s="29">
-        <v>0</v>
-      </c>
-      <c r="D14" s="17">
-        <v>1</v>
-      </c>
-      <c r="E14" s="29">
-        <v>1</v>
-      </c>
-      <c r="F14" s="17">
-        <v>2</v>
-      </c>
-      <c r="G14" s="29">
-        <v>2</v>
-      </c>
-      <c r="H14" s="17">
-        <v>2</v>
-      </c>
-      <c r="I14" s="29">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="16">
+        <v>0</v>
+      </c>
+      <c r="C14" s="28">
+        <v>0</v>
+      </c>
+      <c r="D14" s="16">
+        <v>1</v>
+      </c>
+      <c r="E14" s="28">
+        <v>1</v>
+      </c>
+      <c r="F14" s="16">
+        <v>2</v>
+      </c>
+      <c r="G14" s="28">
+        <v>2</v>
+      </c>
+      <c r="H14" s="16">
+        <v>2</v>
+      </c>
+      <c r="I14" s="28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="17">
-        <v>0</v>
-      </c>
-      <c r="C15" s="29">
-        <v>0</v>
-      </c>
-      <c r="D15" s="17">
-        <v>0</v>
-      </c>
-      <c r="E15" s="29">
-        <v>0</v>
-      </c>
-      <c r="F15" s="17">
-        <v>1</v>
-      </c>
-      <c r="G15" s="29">
-        <v>1</v>
-      </c>
-      <c r="H15" s="17">
-        <v>1</v>
-      </c>
-      <c r="I15" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B15" s="16">
+        <v>0</v>
+      </c>
+      <c r="C15" s="28">
+        <v>0</v>
+      </c>
+      <c r="D15" s="16">
+        <v>0</v>
+      </c>
+      <c r="E15" s="28">
+        <v>0</v>
+      </c>
+      <c r="F15" s="16">
+        <v>1</v>
+      </c>
+      <c r="G15" s="28">
+        <v>1</v>
+      </c>
+      <c r="H15" s="16">
+        <v>1</v>
+      </c>
+      <c r="I15" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="17">
-        <v>0</v>
-      </c>
-      <c r="C16" s="29">
-        <v>0</v>
-      </c>
-      <c r="D16" s="17">
-        <v>0</v>
-      </c>
-      <c r="E16" s="29">
-        <v>0</v>
-      </c>
-      <c r="F16" s="17">
-        <v>0</v>
-      </c>
-      <c r="G16" s="29">
-        <v>0</v>
-      </c>
-      <c r="H16" s="17">
-        <v>1</v>
-      </c>
-      <c r="I16" s="29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="19" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="45" t="s">
+      <c r="B16" s="16">
+        <v>0</v>
+      </c>
+      <c r="C16" s="28">
+        <v>0</v>
+      </c>
+      <c r="D16" s="16">
+        <v>0</v>
+      </c>
+      <c r="E16" s="28">
+        <v>0</v>
+      </c>
+      <c r="F16" s="16">
+        <v>0</v>
+      </c>
+      <c r="G16" s="28">
+        <v>0</v>
+      </c>
+      <c r="H16" s="16">
+        <v>1</v>
+      </c>
+      <c r="I16" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="46"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="46"/>
-      <c r="I17" s="46"/>
-    </row>
-    <row r="18" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="49"/>
+    </row>
+    <row r="18" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="19">
-        <v>0</v>
-      </c>
-      <c r="C18" s="30">
-        <v>2</v>
-      </c>
-      <c r="D18" s="19">
-        <v>0</v>
-      </c>
-      <c r="E18" s="30">
+      <c r="B18" s="18">
+        <v>0</v>
+      </c>
+      <c r="C18" s="29">
+        <v>2</v>
+      </c>
+      <c r="D18" s="18">
+        <v>0</v>
+      </c>
+      <c r="E18" s="29">
         <v>3</v>
       </c>
-      <c r="F18" s="19">
-        <v>0</v>
-      </c>
-      <c r="G18" s="30">
+      <c r="F18" s="18">
+        <v>0</v>
+      </c>
+      <c r="G18" s="29">
         <v>5</v>
       </c>
-      <c r="H18" s="19">
-        <v>0</v>
-      </c>
-      <c r="I18" s="30">
+      <c r="H18" s="18">
+        <v>0</v>
+      </c>
+      <c r="I18" s="29">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="20">
+      <c r="B19" s="19">
         <v>4</v>
       </c>
-      <c r="C19" s="31">
-        <v>2</v>
-      </c>
-      <c r="D19" s="20">
+      <c r="C19" s="30">
+        <v>2</v>
+      </c>
+      <c r="D19" s="19">
         <v>6</v>
       </c>
-      <c r="E19" s="31">
+      <c r="E19" s="30">
         <v>3</v>
       </c>
-      <c r="F19" s="20">
+      <c r="F19" s="19">
         <v>8</v>
       </c>
-      <c r="G19" s="31">
+      <c r="G19" s="30">
         <v>5</v>
       </c>
-      <c r="H19" s="20">
+      <c r="H19" s="19">
         <v>10</v>
       </c>
-      <c r="I19" s="31">
+      <c r="I19" s="30">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="20">
-        <v>2</v>
-      </c>
-      <c r="C20" s="31">
-        <v>2</v>
-      </c>
-      <c r="D20" s="20">
+      <c r="B20" s="19">
+        <v>2</v>
+      </c>
+      <c r="C20" s="30">
+        <v>2</v>
+      </c>
+      <c r="D20" s="19">
         <v>3</v>
       </c>
-      <c r="E20" s="31">
+      <c r="E20" s="30">
         <v>3</v>
       </c>
-      <c r="F20" s="20">
+      <c r="F20" s="19">
         <v>5</v>
       </c>
-      <c r="G20" s="31">
+      <c r="G20" s="30">
         <v>5</v>
       </c>
-      <c r="H20" s="20">
+      <c r="H20" s="19">
         <v>7</v>
       </c>
-      <c r="I20" s="31">
+      <c r="I20" s="30">
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="20">
-        <v>0</v>
-      </c>
-      <c r="C21" s="31">
-        <v>0</v>
-      </c>
-      <c r="D21" s="20">
-        <v>1</v>
-      </c>
-      <c r="E21" s="31">
-        <v>2</v>
-      </c>
-      <c r="F21" s="20">
-        <v>2</v>
-      </c>
-      <c r="G21" s="31">
-        <v>2</v>
-      </c>
-      <c r="H21" s="20">
-        <v>2</v>
-      </c>
-      <c r="I21" s="31">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="19">
+        <v>0</v>
+      </c>
+      <c r="C21" s="30">
+        <v>0</v>
+      </c>
+      <c r="D21" s="19">
+        <v>1</v>
+      </c>
+      <c r="E21" s="30">
+        <v>2</v>
+      </c>
+      <c r="F21" s="19">
+        <v>2</v>
+      </c>
+      <c r="G21" s="30">
+        <v>2</v>
+      </c>
+      <c r="H21" s="19">
+        <v>2</v>
+      </c>
+      <c r="I21" s="30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="21">
-        <v>0</v>
-      </c>
-      <c r="C22" s="32">
-        <v>0</v>
-      </c>
-      <c r="D22" s="21">
-        <v>1</v>
-      </c>
-      <c r="E22" s="32">
-        <v>1</v>
-      </c>
-      <c r="F22" s="21">
-        <v>2</v>
-      </c>
-      <c r="G22" s="32">
-        <v>2</v>
-      </c>
-      <c r="H22" s="21">
+      <c r="B22" s="20">
+        <v>0</v>
+      </c>
+      <c r="C22" s="31">
+        <v>0</v>
+      </c>
+      <c r="D22" s="20">
+        <v>1</v>
+      </c>
+      <c r="E22" s="31">
+        <v>1</v>
+      </c>
+      <c r="F22" s="20">
+        <v>2</v>
+      </c>
+      <c r="G22" s="31">
+        <v>2</v>
+      </c>
+      <c r="H22" s="20">
         <v>3</v>
       </c>
-      <c r="I22" s="32">
+      <c r="I22" s="31">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="20">
-        <v>0</v>
-      </c>
-      <c r="C23" s="31">
-        <v>0</v>
-      </c>
-      <c r="D23" s="20">
-        <v>0</v>
-      </c>
-      <c r="E23" s="31">
-        <v>0</v>
-      </c>
-      <c r="F23" s="20">
+      <c r="B23" s="19">
+        <v>0</v>
+      </c>
+      <c r="C23" s="30">
+        <v>0</v>
+      </c>
+      <c r="D23" s="19">
+        <v>0</v>
+      </c>
+      <c r="E23" s="30">
+        <v>0</v>
+      </c>
+      <c r="F23" s="19">
         <v>4</v>
       </c>
-      <c r="G23" s="31">
+      <c r="G23" s="30">
         <v>4</v>
       </c>
-      <c r="H23" s="20">
+      <c r="H23" s="19">
         <v>6</v>
       </c>
-      <c r="I23" s="31">
+      <c r="I23" s="30">
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A24" s="47" t="s">
-        <v>2</v>
-      </c>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="48"/>
-    </row>
-    <row r="25" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A24" s="50" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" s="51"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="51"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="51"/>
+      <c r="H24" s="51"/>
+      <c r="I24" s="51"/>
+    </row>
+    <row r="25" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B25" s="19">
-        <v>0</v>
-      </c>
-      <c r="C25" s="30">
-        <v>1</v>
-      </c>
-      <c r="D25" s="19">
-        <v>0</v>
-      </c>
-      <c r="E25" s="30">
-        <v>2</v>
-      </c>
-      <c r="F25" s="19">
-        <v>0</v>
-      </c>
-      <c r="G25" s="30">
+      <c r="B25" s="18">
+        <v>0</v>
+      </c>
+      <c r="C25" s="29">
+        <v>1</v>
+      </c>
+      <c r="D25" s="18">
+        <v>0</v>
+      </c>
+      <c r="E25" s="29">
+        <v>2</v>
+      </c>
+      <c r="F25" s="18">
+        <v>0</v>
+      </c>
+      <c r="G25" s="29">
         <v>3</v>
       </c>
-      <c r="H25" s="19">
-        <v>0</v>
-      </c>
-      <c r="I25" s="30">
+      <c r="H25" s="18">
+        <v>0</v>
+      </c>
+      <c r="I25" s="29">
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B26" s="20">
-        <v>1</v>
-      </c>
-      <c r="C26" s="31">
-        <v>1</v>
-      </c>
-      <c r="D26" s="20">
-        <v>1</v>
-      </c>
-      <c r="E26" s="31">
-        <v>1</v>
-      </c>
-      <c r="F26" s="20">
-        <v>1</v>
-      </c>
-      <c r="G26" s="31">
-        <v>1</v>
-      </c>
-      <c r="H26" s="20">
-        <v>2</v>
-      </c>
-      <c r="I26" s="31">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="19">
+        <v>1</v>
+      </c>
+      <c r="C26" s="30">
+        <v>1</v>
+      </c>
+      <c r="D26" s="19">
+        <v>1</v>
+      </c>
+      <c r="E26" s="30">
+        <v>1</v>
+      </c>
+      <c r="F26" s="19">
+        <v>1</v>
+      </c>
+      <c r="G26" s="30">
+        <v>1</v>
+      </c>
+      <c r="H26" s="19">
+        <v>2</v>
+      </c>
+      <c r="I26" s="30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="20">
-        <v>2</v>
-      </c>
-      <c r="C27" s="31">
-        <v>2</v>
-      </c>
-      <c r="D27" s="20">
+      <c r="B27" s="19">
+        <v>2</v>
+      </c>
+      <c r="C27" s="30">
+        <v>2</v>
+      </c>
+      <c r="D27" s="19">
         <v>4</v>
       </c>
-      <c r="E27" s="31">
+      <c r="E27" s="30">
         <v>3</v>
       </c>
-      <c r="F27" s="20">
+      <c r="F27" s="19">
         <v>8</v>
       </c>
-      <c r="G27" s="31">
+      <c r="G27" s="30">
         <v>6</v>
       </c>
-      <c r="H27" s="20">
+      <c r="H27" s="19">
         <v>12</v>
       </c>
-      <c r="I27" s="31">
+      <c r="I27" s="30">
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B28" s="20">
-        <v>1</v>
-      </c>
-      <c r="C28" s="31">
-        <v>1</v>
-      </c>
-      <c r="D28" s="20">
-        <v>1</v>
-      </c>
-      <c r="E28" s="31">
-        <v>1</v>
-      </c>
-      <c r="F28" s="20">
-        <v>1</v>
-      </c>
-      <c r="G28" s="31">
-        <v>1</v>
-      </c>
-      <c r="H28" s="20">
-        <v>1</v>
-      </c>
-      <c r="I28" s="31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="19">
+        <v>1</v>
+      </c>
+      <c r="C28" s="30">
+        <v>1</v>
+      </c>
+      <c r="D28" s="19">
+        <v>1</v>
+      </c>
+      <c r="E28" s="30">
+        <v>1</v>
+      </c>
+      <c r="F28" s="19">
+        <v>1</v>
+      </c>
+      <c r="G28" s="30">
+        <v>1</v>
+      </c>
+      <c r="H28" s="19">
+        <v>1</v>
+      </c>
+      <c r="I28" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="20">
-        <v>1</v>
-      </c>
-      <c r="C29" s="31">
-        <v>1</v>
-      </c>
-      <c r="D29" s="20">
-        <v>1</v>
-      </c>
-      <c r="E29" s="31">
-        <v>1</v>
-      </c>
-      <c r="F29" s="20">
-        <v>2</v>
-      </c>
-      <c r="G29" s="31">
-        <v>2</v>
-      </c>
-      <c r="H29" s="20">
+      <c r="B29" s="19">
+        <v>1</v>
+      </c>
+      <c r="C29" s="30">
+        <v>1</v>
+      </c>
+      <c r="D29" s="19">
+        <v>1</v>
+      </c>
+      <c r="E29" s="30">
+        <v>1</v>
+      </c>
+      <c r="F29" s="19">
+        <v>2</v>
+      </c>
+      <c r="G29" s="30">
+        <v>2</v>
+      </c>
+      <c r="H29" s="19">
         <v>3</v>
       </c>
-      <c r="I29" s="31">
+      <c r="I29" s="30">
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="20">
-        <v>1</v>
-      </c>
-      <c r="C30" s="31">
-        <v>1</v>
-      </c>
-      <c r="D30" s="20">
-        <v>1</v>
-      </c>
-      <c r="E30" s="31">
-        <v>1</v>
-      </c>
-      <c r="F30" s="20">
-        <v>1</v>
-      </c>
-      <c r="G30" s="31">
-        <v>1</v>
-      </c>
-      <c r="H30" s="20">
-        <v>1</v>
-      </c>
-      <c r="I30" s="31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="19">
+        <v>1</v>
+      </c>
+      <c r="C30" s="30">
+        <v>1</v>
+      </c>
+      <c r="D30" s="19">
+        <v>1</v>
+      </c>
+      <c r="E30" s="30">
+        <v>1</v>
+      </c>
+      <c r="F30" s="19">
+        <v>1</v>
+      </c>
+      <c r="G30" s="30">
+        <v>1</v>
+      </c>
+      <c r="H30" s="19">
+        <v>1</v>
+      </c>
+      <c r="I30" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="20">
-        <v>1</v>
-      </c>
-      <c r="C31" s="31">
-        <v>1</v>
-      </c>
-      <c r="D31" s="20">
-        <v>1</v>
-      </c>
-      <c r="E31" s="31">
-        <v>1</v>
-      </c>
-      <c r="F31" s="20">
-        <v>1</v>
-      </c>
-      <c r="G31" s="31">
-        <v>1</v>
-      </c>
-      <c r="H31" s="20">
-        <v>2</v>
-      </c>
-      <c r="I31" s="31">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B31" s="19">
+        <v>1</v>
+      </c>
+      <c r="C31" s="30">
+        <v>1</v>
+      </c>
+      <c r="D31" s="19">
+        <v>1</v>
+      </c>
+      <c r="E31" s="30">
+        <v>1</v>
+      </c>
+      <c r="F31" s="19">
+        <v>1</v>
+      </c>
+      <c r="G31" s="30">
+        <v>1</v>
+      </c>
+      <c r="H31" s="19">
+        <v>2</v>
+      </c>
+      <c r="I31" s="30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B32" s="22">
-        <v>2</v>
-      </c>
-      <c r="C32" s="33">
-        <v>2</v>
-      </c>
-      <c r="D32" s="22">
+      <c r="B32" s="21">
+        <v>2</v>
+      </c>
+      <c r="C32" s="32">
+        <v>2</v>
+      </c>
+      <c r="D32" s="21">
         <v>4</v>
       </c>
-      <c r="E32" s="33">
+      <c r="E32" s="32">
         <v>4</v>
       </c>
-      <c r="F32" s="22">
+      <c r="F32" s="21">
         <v>4</v>
       </c>
-      <c r="G32" s="33">
+      <c r="G32" s="32">
         <v>4</v>
       </c>
-      <c r="H32" s="22">
+      <c r="H32" s="21">
         <v>8</v>
       </c>
-      <c r="I32" s="33">
+      <c r="I32" s="32">
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B33" s="23">
-        <v>2</v>
-      </c>
-      <c r="C33" s="34">
-        <v>2</v>
-      </c>
-      <c r="D33" s="23">
+      <c r="B33" s="22">
+        <v>2</v>
+      </c>
+      <c r="C33" s="33">
+        <v>2</v>
+      </c>
+      <c r="D33" s="22">
         <v>3</v>
       </c>
-      <c r="E33" s="34">
+      <c r="E33" s="33">
         <v>3</v>
       </c>
-      <c r="F33" s="23">
+      <c r="F33" s="22">
         <v>6</v>
       </c>
-      <c r="G33" s="34">
+      <c r="G33" s="33">
         <v>6</v>
       </c>
-      <c r="H33" s="23">
+      <c r="H33" s="22">
         <v>10</v>
       </c>
-      <c r="I33" s="34">
+      <c r="I33" s="33">
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="50" t="s">
+    <row r="34" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="B34" s="51">
-        <v>0</v>
-      </c>
-      <c r="C34" s="52">
-        <v>0</v>
-      </c>
-      <c r="D34" s="51">
-        <v>0</v>
-      </c>
-      <c r="E34" s="52">
-        <v>0</v>
-      </c>
-      <c r="F34" s="51">
-        <v>1</v>
-      </c>
-      <c r="G34" s="52">
-        <v>1</v>
-      </c>
-      <c r="H34" s="51">
-        <v>2</v>
-      </c>
-      <c r="I34" s="52">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B34" s="38">
+        <v>0</v>
+      </c>
+      <c r="C34" s="39">
+        <v>0</v>
+      </c>
+      <c r="D34" s="38">
+        <v>0</v>
+      </c>
+      <c r="E34" s="39">
+        <v>0</v>
+      </c>
+      <c r="F34" s="38">
+        <v>1</v>
+      </c>
+      <c r="G34" s="39">
+        <v>1</v>
+      </c>
+      <c r="H34" s="38">
+        <v>2</v>
+      </c>
+      <c r="I34" s="39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B35" s="22">
-        <v>0</v>
-      </c>
-      <c r="C35" s="33">
-        <v>0</v>
-      </c>
-      <c r="D35" s="22">
-        <v>1</v>
-      </c>
-      <c r="E35" s="33">
-        <v>1</v>
-      </c>
-      <c r="F35" s="22">
-        <v>2</v>
-      </c>
-      <c r="G35" s="33">
-        <v>2</v>
-      </c>
-      <c r="H35" s="22">
+      <c r="B35" s="21">
+        <v>0</v>
+      </c>
+      <c r="C35" s="32">
+        <v>0</v>
+      </c>
+      <c r="D35" s="21">
+        <v>1</v>
+      </c>
+      <c r="E35" s="32">
+        <v>1</v>
+      </c>
+      <c r="F35" s="21">
+        <v>2</v>
+      </c>
+      <c r="G35" s="32">
+        <v>2</v>
+      </c>
+      <c r="H35" s="21">
         <v>3</v>
       </c>
-      <c r="I35" s="33">
+      <c r="I35" s="32">
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B36" s="24">
+      <c r="B36" s="23">
         <f t="shared" ref="B36:I36" si="0">SUM(B14:B35)</f>
         <v>17</v>
       </c>
-      <c r="C36" s="35">
+      <c r="C36" s="34">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="D36" s="24">
+      <c r="D36" s="23">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="E36" s="35">
+      <c r="E36" s="34">
         <f>SUM(E14:E35)</f>
         <v>31</v>
       </c>
-      <c r="F36" s="24">
+      <c r="F36" s="23">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="G36" s="35">
+      <c r="G36" s="34">
         <f>SUM(G14:G35)</f>
         <v>54</v>
       </c>
-      <c r="H36" s="24">
+      <c r="H36" s="23">
         <f t="shared" si="0"/>
         <v>76</v>
       </c>
-      <c r="I36" s="35">
+      <c r="I36" s="34">
         <f t="shared" si="0"/>
         <v>84</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="36" t="s">
+    <row r="38" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="35" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="49" t="s">
+    <row r="39" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="B39" s="49"/>
-      <c r="C39" s="49"/>
-      <c r="D39" s="49"/>
-      <c r="E39" s="49"/>
-      <c r="F39" s="49"/>
-      <c r="G39" s="49"/>
-      <c r="H39" s="49"/>
-      <c r="I39" s="49"/>
-    </row>
-    <row r="40" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="49" t="s">
+      <c r="B39" s="40"/>
+      <c r="C39" s="40"/>
+      <c r="D39" s="40"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="40"/>
+      <c r="G39" s="40"/>
+      <c r="H39" s="40"/>
+      <c r="I39" s="40"/>
+    </row>
+    <row r="40" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="B40" s="49"/>
-      <c r="C40" s="49"/>
-      <c r="D40" s="49"/>
-      <c r="E40" s="49"/>
-      <c r="F40" s="49"/>
-      <c r="G40" s="49"/>
-      <c r="H40" s="49"/>
-      <c r="I40" s="49"/>
-    </row>
-    <row r="41" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="49" t="s">
+      <c r="B40" s="40"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="40"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="40"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="40"/>
+    </row>
+    <row r="41" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="49"/>
-      <c r="C41" s="49"/>
-      <c r="D41" s="49"/>
-      <c r="E41" s="49"/>
-      <c r="F41" s="49"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="49"/>
-      <c r="I41" s="49"/>
-    </row>
-    <row r="42" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="49" t="s">
+      <c r="B41" s="40"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="40"/>
+      <c r="E41" s="40"/>
+      <c r="F41" s="40"/>
+      <c r="G41" s="40"/>
+      <c r="H41" s="40"/>
+      <c r="I41" s="40"/>
+    </row>
+    <row r="42" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="49"/>
-      <c r="C42" s="49"/>
-      <c r="D42" s="49"/>
-      <c r="E42" s="49"/>
-      <c r="F42" s="49"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="49"/>
-      <c r="I42" s="49"/>
-    </row>
-    <row r="43" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="49"/>
-      <c r="B43" s="49"/>
-      <c r="C43" s="49"/>
-      <c r="D43" s="49"/>
-      <c r="E43" s="49"/>
-      <c r="F43" s="49"/>
-      <c r="G43" s="49"/>
-      <c r="H43" s="49"/>
-      <c r="I43" s="49"/>
-    </row>
-    <row r="44" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="49"/>
-      <c r="B44" s="49"/>
-      <c r="C44" s="49"/>
-      <c r="D44" s="49"/>
-      <c r="E44" s="49"/>
-      <c r="F44" s="49"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="49"/>
-      <c r="I44" s="49"/>
-    </row>
-    <row r="45" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="49"/>
-      <c r="B45" s="49"/>
-      <c r="C45" s="49"/>
-      <c r="D45" s="49"/>
-      <c r="E45" s="49"/>
-      <c r="F45" s="49"/>
-      <c r="G45" s="49"/>
-      <c r="H45" s="49"/>
-      <c r="I45" s="49"/>
-    </row>
-    <row r="46" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="49"/>
-      <c r="B46" s="49"/>
-      <c r="C46" s="49"/>
-      <c r="D46" s="49"/>
-      <c r="E46" s="49"/>
-      <c r="F46" s="49"/>
-      <c r="G46" s="49"/>
-      <c r="H46" s="49"/>
-      <c r="I46" s="49"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="40"/>
+      <c r="F42" s="40"/>
+      <c r="G42" s="40"/>
+      <c r="H42" s="40"/>
+      <c r="I42" s="40"/>
+    </row>
+    <row r="43" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="40"/>
+      <c r="B43" s="40"/>
+      <c r="C43" s="40"/>
+      <c r="D43" s="40"/>
+      <c r="E43" s="40"/>
+      <c r="F43" s="40"/>
+      <c r="G43" s="40"/>
+      <c r="H43" s="40"/>
+      <c r="I43" s="40"/>
+    </row>
+    <row r="44" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="40"/>
+      <c r="B44" s="40"/>
+      <c r="C44" s="40"/>
+      <c r="D44" s="40"/>
+      <c r="E44" s="40"/>
+      <c r="F44" s="40"/>
+      <c r="G44" s="40"/>
+      <c r="H44" s="40"/>
+      <c r="I44" s="40"/>
+    </row>
+    <row r="45" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="40"/>
+      <c r="B45" s="40"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="40"/>
+      <c r="I45" s="40"/>
+    </row>
+    <row r="46" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="40"/>
+      <c r="B46" s="40"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="40"/>
+      <c r="E46" s="40"/>
+      <c r="F46" s="40"/>
+      <c r="G46" s="40"/>
+      <c r="H46" s="40"/>
+      <c r="I46" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A1:I5"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A24:I24"/>
     <mergeCell ref="A44:I44"/>
     <mergeCell ref="A45:I45"/>
     <mergeCell ref="A46:I46"/>
@@ -2099,11 +2074,6 @@
     <mergeCell ref="A41:I41"/>
     <mergeCell ref="A42:I42"/>
     <mergeCell ref="A43:I43"/>
-    <mergeCell ref="A1:I5"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A24:I24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="300" r:id="rId1"/>

</xml_diff>